<commit_message>
feat(nandu): info del certamen nacional 2026
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/files/nacional/nandu/PlanillaNacional.xlsx
+++ b/public/files/nacional/nandu/PlanillaNacional.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marit\Dropbox\Ñandú\2024\Competencias_nandu\Nacional\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marita\Dropbox\Ñandú\2026\Competencias_Ñandu\06_nacional\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC46C32F-BC85-4BDC-83D3-AC3730B995CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5207209B-0185-41F5-AD0F-0554C5A33FA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$Q$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$P$28</definedName>
   </definedNames>
   <calcPr calcId="144525"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>N°</t>
   </si>
@@ -54,9 +54,6 @@
   </si>
   <si>
     <t>DNI</t>
-  </si>
-  <si>
-    <t>Sexo</t>
   </si>
   <si>
     <t>Tipo (*)</t>
@@ -170,10 +167,10 @@
     </r>
   </si>
   <si>
-    <t>Vianda 23</t>
+    <t xml:space="preserve">Provincia </t>
   </si>
   <si>
-    <t>Provincia</t>
+    <t>Género</t>
   </si>
 </sst>
 </file>
@@ -183,7 +180,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -194,40 +191,38 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
-      <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -315,7 +310,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -358,26 +353,23 @@
     <xf numFmtId="3" fontId="6" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -604,28 +596,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5546875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P30"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" customWidth="1"/>
-    <col min="2" max="2" width="12.109375" style="20" customWidth="1"/>
-    <col min="3" max="3" width="20.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="14.44140625" customWidth="1"/>
-    <col min="6" max="6" width="8" style="24" customWidth="1"/>
-    <col min="7" max="7" width="23.5546875" customWidth="1"/>
-    <col min="8" max="8" width="22.88671875" customWidth="1"/>
-    <col min="9" max="9" width="14.109375" customWidth="1"/>
-    <col min="10" max="10" width="7.88671875" customWidth="1"/>
-    <col min="11" max="11" width="8.33203125" customWidth="1"/>
+    <col min="1" max="1" width="4.7265625" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" style="19" customWidth="1"/>
+    <col min="3" max="3" width="20.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="14.453125" customWidth="1"/>
+    <col min="6" max="6" width="8" style="23" customWidth="1"/>
+    <col min="7" max="7" width="23.54296875" customWidth="1"/>
+    <col min="8" max="8" width="22.81640625" customWidth="1"/>
+    <col min="9" max="9" width="14.1796875" customWidth="1"/>
+    <col min="10" max="10" width="7.81640625" customWidth="1"/>
+    <col min="11" max="11" width="8.26953125" customWidth="1"/>
     <col min="12" max="12" width="8" customWidth="1"/>
-    <col min="13" max="13" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.44140625" customWidth="1"/>
-    <col min="15" max="15" width="9.44140625" customWidth="1"/>
-    <col min="16" max="16" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.453125" customWidth="1"/>
+    <col min="15" max="15" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="17" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" s="16" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
@@ -639,7 +630,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="14" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F1" s="14" t="s">
         <v>4</v>
@@ -654,531 +645,502 @@
         <v>7</v>
       </c>
       <c r="J1" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="K1" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="14" t="s">
+      <c r="L1" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="14" t="s">
+      <c r="M1" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="14" t="s">
+      <c r="O1" s="14" t="s">
         <v>12</v>
-      </c>
-      <c r="N1" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="O1" s="16" t="s">
-        <v>16</v>
       </c>
       <c r="P1" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="Q1" s="14" t="s">
-        <v>14</v>
-      </c>
     </row>
-    <row r="2" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
       <c r="I2" s="7"/>
-      <c r="J2" s="26"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="26"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
       <c r="M2" s="4"/>
-      <c r="N2" s="26"/>
-      <c r="O2" s="26"/>
-      <c r="P2" s="5"/>
-      <c r="Q2" s="6"/>
+      <c r="N2" s="25"/>
+      <c r="O2" s="5"/>
+      <c r="P2" s="6"/>
     </row>
-    <row r="3" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="25"/>
-      <c r="H3" s="25"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
       <c r="I3" s="7"/>
-      <c r="J3" s="26"/>
-      <c r="K3" s="26"/>
-      <c r="L3" s="26"/>
+      <c r="J3" s="25"/>
+      <c r="K3" s="25"/>
+      <c r="L3" s="25"/>
       <c r="M3" s="4"/>
-      <c r="N3" s="26"/>
-      <c r="O3" s="26"/>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="6"/>
+      <c r="N3" s="25"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="6"/>
     </row>
-    <row r="4" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" s="1"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="25"/>
-      <c r="H4" s="25"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
       <c r="I4" s="7"/>
-      <c r="J4" s="26"/>
-      <c r="K4" s="26"/>
-      <c r="L4" s="26"/>
+      <c r="J4" s="25"/>
+      <c r="K4" s="25"/>
+      <c r="L4" s="25"/>
       <c r="M4" s="4"/>
-      <c r="N4" s="26"/>
-      <c r="O4" s="26"/>
-      <c r="P4" s="5"/>
-      <c r="Q4" s="6"/>
+      <c r="N4" s="25"/>
+      <c r="O4" s="5"/>
+      <c r="P4" s="6"/>
     </row>
-    <row r="5" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="1"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="25"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
       <c r="I5" s="7"/>
-      <c r="J5" s="26"/>
-      <c r="K5" s="26"/>
-      <c r="L5" s="26"/>
+      <c r="J5" s="25"/>
+      <c r="K5" s="25"/>
+      <c r="L5" s="25"/>
       <c r="M5" s="4"/>
-      <c r="N5" s="26"/>
-      <c r="O5" s="26"/>
-      <c r="P5" s="5"/>
-      <c r="Q5" s="6"/>
+      <c r="N5" s="25"/>
+      <c r="O5" s="5"/>
+      <c r="P5" s="6"/>
     </row>
-    <row r="6" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
       <c r="B6" s="1"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24"/>
       <c r="I6" s="7"/>
-      <c r="J6" s="26"/>
-      <c r="K6" s="26"/>
-      <c r="L6" s="26"/>
+      <c r="J6" s="25"/>
+      <c r="K6" s="25"/>
+      <c r="L6" s="25"/>
       <c r="M6" s="4"/>
-      <c r="N6" s="26"/>
-      <c r="O6" s="26"/>
-      <c r="P6" s="5"/>
-      <c r="Q6" s="6"/>
+      <c r="N6" s="25"/>
+      <c r="O6" s="5"/>
+      <c r="P6" s="6"/>
     </row>
-    <row r="7" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" s="1"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="25"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="24"/>
       <c r="I7" s="7"/>
-      <c r="J7" s="26"/>
-      <c r="K7" s="26"/>
-      <c r="L7" s="26"/>
+      <c r="J7" s="25"/>
+      <c r="K7" s="25"/>
+      <c r="L7" s="25"/>
       <c r="M7" s="4"/>
-      <c r="N7" s="26"/>
-      <c r="O7" s="26"/>
-      <c r="P7" s="5"/>
-      <c r="Q7" s="6"/>
+      <c r="N7" s="25"/>
+      <c r="O7" s="5"/>
+      <c r="P7" s="6"/>
     </row>
-    <row r="8" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="1"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="19"/>
-      <c r="F8" s="22"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="25"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="24"/>
+      <c r="H8" s="24"/>
       <c r="I8" s="7"/>
-      <c r="J8" s="26"/>
-      <c r="K8" s="26"/>
-      <c r="L8" s="26"/>
+      <c r="J8" s="25"/>
+      <c r="K8" s="25"/>
+      <c r="L8" s="25"/>
       <c r="M8" s="4"/>
-      <c r="N8" s="26"/>
-      <c r="O8" s="26"/>
-      <c r="P8" s="5"/>
-      <c r="Q8" s="6"/>
+      <c r="N8" s="25"/>
+      <c r="O8" s="5"/>
+      <c r="P8" s="6"/>
     </row>
-    <row r="9" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="1"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="25"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="24"/>
       <c r="I9" s="7"/>
-      <c r="J9" s="26"/>
-      <c r="K9" s="26"/>
-      <c r="L9" s="26"/>
+      <c r="J9" s="25"/>
+      <c r="K9" s="25"/>
+      <c r="L9" s="25"/>
       <c r="M9" s="4"/>
-      <c r="N9" s="26"/>
-      <c r="O9" s="26"/>
-      <c r="P9" s="5"/>
-      <c r="Q9" s="6"/>
+      <c r="N9" s="25"/>
+      <c r="O9" s="5"/>
+      <c r="P9" s="6"/>
     </row>
-    <row r="10" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="1"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="25"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
       <c r="I10" s="7"/>
-      <c r="J10" s="26"/>
-      <c r="K10" s="26"/>
-      <c r="L10" s="26"/>
+      <c r="J10" s="25"/>
+      <c r="K10" s="25"/>
+      <c r="L10" s="25"/>
       <c r="M10" s="4"/>
-      <c r="N10" s="26"/>
-      <c r="O10" s="26"/>
-      <c r="P10" s="5"/>
-      <c r="Q10" s="6"/>
+      <c r="N10" s="25"/>
+      <c r="O10" s="5"/>
+      <c r="P10" s="6"/>
     </row>
-    <row r="11" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="1"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="22"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="25"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="24"/>
+      <c r="H11" s="24"/>
       <c r="I11" s="7"/>
-      <c r="J11" s="26"/>
-      <c r="K11" s="26"/>
-      <c r="L11" s="26"/>
+      <c r="J11" s="25"/>
+      <c r="K11" s="25"/>
+      <c r="L11" s="25"/>
       <c r="M11" s="4"/>
-      <c r="N11" s="26"/>
-      <c r="O11" s="26"/>
-      <c r="P11" s="5"/>
-      <c r="Q11" s="6"/>
+      <c r="N11" s="25"/>
+      <c r="O11" s="5"/>
+      <c r="P11" s="6"/>
     </row>
-    <row r="12" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="1"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="25"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="24"/>
       <c r="I12" s="7"/>
-      <c r="J12" s="26"/>
-      <c r="K12" s="26"/>
-      <c r="L12" s="26"/>
+      <c r="J12" s="25"/>
+      <c r="K12" s="25"/>
+      <c r="L12" s="25"/>
       <c r="M12" s="4"/>
-      <c r="N12" s="26"/>
-      <c r="O12" s="26"/>
-      <c r="P12" s="5"/>
-      <c r="Q12" s="6"/>
+      <c r="N12" s="25"/>
+      <c r="O12" s="5"/>
+      <c r="P12" s="6"/>
     </row>
-    <row r="13" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
       <c r="B13" s="1"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="25"/>
-      <c r="H13" s="25"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="24"/>
       <c r="I13" s="7"/>
-      <c r="J13" s="26"/>
-      <c r="K13" s="26"/>
-      <c r="L13" s="26"/>
+      <c r="J13" s="25"/>
+      <c r="K13" s="25"/>
+      <c r="L13" s="25"/>
       <c r="M13" s="4"/>
-      <c r="N13" s="26"/>
-      <c r="O13" s="26"/>
-      <c r="P13" s="5"/>
-      <c r="Q13" s="6"/>
+      <c r="N13" s="25"/>
+      <c r="O13" s="5"/>
+      <c r="P13" s="6"/>
     </row>
-    <row r="14" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="1"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="25"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="24"/>
       <c r="I14" s="7"/>
-      <c r="J14" s="26"/>
-      <c r="K14" s="26"/>
-      <c r="L14" s="26"/>
+      <c r="J14" s="25"/>
+      <c r="K14" s="25"/>
+      <c r="L14" s="25"/>
       <c r="M14" s="4"/>
-      <c r="N14" s="26"/>
-      <c r="O14" s="26"/>
-      <c r="P14" s="5"/>
-      <c r="Q14" s="6"/>
+      <c r="N14" s="25"/>
+      <c r="O14" s="5"/>
+      <c r="P14" s="6"/>
     </row>
-    <row r="15" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="1"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="25"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="24"/>
+      <c r="H15" s="24"/>
       <c r="I15" s="7"/>
-      <c r="J15" s="26"/>
-      <c r="K15" s="26"/>
-      <c r="L15" s="26"/>
+      <c r="J15" s="25"/>
+      <c r="K15" s="25"/>
+      <c r="L15" s="25"/>
       <c r="M15" s="4"/>
-      <c r="N15" s="26"/>
-      <c r="O15" s="26"/>
-      <c r="P15" s="5"/>
-      <c r="Q15" s="6"/>
+      <c r="N15" s="25"/>
+      <c r="O15" s="5"/>
+      <c r="P15" s="6"/>
     </row>
-    <row r="16" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="1"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="25"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="21"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
       <c r="I16" s="7"/>
-      <c r="J16" s="26"/>
-      <c r="K16" s="26"/>
-      <c r="L16" s="26"/>
+      <c r="J16" s="25"/>
+      <c r="K16" s="25"/>
+      <c r="L16" s="25"/>
       <c r="M16" s="4"/>
-      <c r="N16" s="26"/>
-      <c r="O16" s="26"/>
-      <c r="P16" s="5"/>
-      <c r="Q16" s="6"/>
+      <c r="N16" s="25"/>
+      <c r="O16" s="5"/>
+      <c r="P16" s="6"/>
     </row>
-    <row r="17" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
       <c r="B17" s="1"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="25"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="21"/>
+      <c r="G17" s="24"/>
+      <c r="H17" s="24"/>
       <c r="I17" s="7"/>
-      <c r="J17" s="26"/>
-      <c r="K17" s="26"/>
-      <c r="L17" s="26"/>
+      <c r="J17" s="25"/>
+      <c r="K17" s="25"/>
+      <c r="L17" s="25"/>
       <c r="M17" s="4"/>
-      <c r="N17" s="26"/>
-      <c r="O17" s="26"/>
-      <c r="P17" s="5"/>
-      <c r="Q17" s="6"/>
+      <c r="N17" s="25"/>
+      <c r="O17" s="5"/>
+      <c r="P17" s="6"/>
     </row>
-    <row r="18" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
       <c r="B18" s="1"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="25"/>
-      <c r="H18" s="25"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="24"/>
       <c r="I18" s="7"/>
-      <c r="J18" s="26"/>
-      <c r="K18" s="26"/>
-      <c r="L18" s="26"/>
+      <c r="J18" s="25"/>
+      <c r="K18" s="25"/>
+      <c r="L18" s="25"/>
       <c r="M18" s="4"/>
-      <c r="N18" s="26"/>
-      <c r="O18" s="26"/>
-      <c r="P18" s="5"/>
-      <c r="Q18" s="6"/>
+      <c r="N18" s="25"/>
+      <c r="O18" s="5"/>
+      <c r="P18" s="6"/>
     </row>
-    <row r="19" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="1"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="25"/>
-      <c r="H19" s="25"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="24"/>
+      <c r="H19" s="24"/>
       <c r="I19" s="7"/>
-      <c r="J19" s="26"/>
-      <c r="K19" s="26"/>
-      <c r="L19" s="26"/>
+      <c r="J19" s="25"/>
+      <c r="K19" s="25"/>
+      <c r="L19" s="25"/>
       <c r="M19" s="4"/>
-      <c r="N19" s="26"/>
-      <c r="O19" s="26"/>
-      <c r="P19" s="5"/>
-      <c r="Q19" s="6"/>
+      <c r="N19" s="25"/>
+      <c r="O19" s="5"/>
+      <c r="P19" s="6"/>
     </row>
-    <row r="20" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="1"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="25"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="24"/>
       <c r="I20" s="7"/>
-      <c r="J20" s="26"/>
-      <c r="K20" s="26"/>
-      <c r="L20" s="26"/>
+      <c r="J20" s="25"/>
+      <c r="K20" s="25"/>
+      <c r="L20" s="25"/>
       <c r="M20" s="4"/>
-      <c r="N20" s="26"/>
-      <c r="O20" s="26"/>
-      <c r="P20" s="5"/>
-      <c r="Q20" s="6"/>
+      <c r="N20" s="25"/>
+      <c r="O20" s="5"/>
+      <c r="P20" s="6"/>
     </row>
-    <row r="21" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="1"/>
-      <c r="C21" s="19"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="25"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="24"/>
       <c r="I21" s="7"/>
-      <c r="J21" s="26"/>
-      <c r="K21" s="26"/>
-      <c r="L21" s="26"/>
+      <c r="J21" s="25"/>
+      <c r="K21" s="25"/>
+      <c r="L21" s="25"/>
       <c r="M21" s="4"/>
-      <c r="N21" s="26"/>
-      <c r="O21" s="26"/>
-      <c r="P21" s="5"/>
-      <c r="Q21" s="6"/>
+      <c r="N21" s="25"/>
+      <c r="O21" s="5"/>
+      <c r="P21" s="6"/>
     </row>
-    <row r="22" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="1"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="25"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="18"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
       <c r="I22" s="7"/>
-      <c r="J22" s="26"/>
-      <c r="K22" s="26"/>
-      <c r="L22" s="26"/>
+      <c r="J22" s="25"/>
+      <c r="K22" s="25"/>
+      <c r="L22" s="25"/>
       <c r="M22" s="4"/>
-      <c r="N22" s="26"/>
-      <c r="O22" s="26"/>
-      <c r="P22" s="5"/>
-      <c r="Q22" s="6"/>
+      <c r="N22" s="25"/>
+      <c r="O22" s="5"/>
+      <c r="P22" s="6"/>
     </row>
-    <row r="23" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
       <c r="B23" s="1"/>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="25"/>
-      <c r="H23" s="25"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="24"/>
       <c r="I23" s="7"/>
-      <c r="J23" s="26"/>
-      <c r="K23" s="26"/>
-      <c r="L23" s="26"/>
+      <c r="J23" s="25"/>
+      <c r="K23" s="25"/>
+      <c r="L23" s="25"/>
       <c r="M23" s="4"/>
-      <c r="N23" s="26"/>
-      <c r="O23" s="26"/>
-      <c r="P23" s="5"/>
-      <c r="Q23" s="6"/>
+      <c r="N23" s="25"/>
+      <c r="O23" s="5"/>
+      <c r="P23" s="6"/>
     </row>
-    <row r="24" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="1"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="22"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="25"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="24"/>
+      <c r="H24" s="24"/>
       <c r="I24" s="7"/>
-      <c r="J24" s="26"/>
-      <c r="K24" s="26"/>
-      <c r="L24" s="26"/>
+      <c r="J24" s="25"/>
+      <c r="K24" s="25"/>
+      <c r="L24" s="25"/>
       <c r="M24" s="4"/>
-      <c r="N24" s="26"/>
-      <c r="O24" s="26"/>
-      <c r="P24" s="5"/>
-      <c r="Q24" s="6"/>
+      <c r="N24" s="25"/>
+      <c r="O24" s="5"/>
+      <c r="P24" s="6"/>
     </row>
-    <row r="25" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="1"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="25"/>
-      <c r="H25" s="25"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="21"/>
+      <c r="G25" s="24"/>
+      <c r="H25" s="24"/>
       <c r="I25" s="7"/>
-      <c r="J25" s="26"/>
-      <c r="K25" s="26"/>
-      <c r="L25" s="26"/>
+      <c r="J25" s="25"/>
+      <c r="K25" s="25"/>
+      <c r="L25" s="25"/>
       <c r="M25" s="4"/>
-      <c r="N25" s="26"/>
-      <c r="O25" s="26"/>
-      <c r="P25" s="5"/>
-      <c r="Q25" s="6"/>
+      <c r="N25" s="25"/>
+      <c r="O25" s="5"/>
+      <c r="P25" s="6"/>
     </row>
-    <row r="26" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3"/>
       <c r="B26" s="1"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="25"/>
-      <c r="H26" s="25"/>
-      <c r="I26" s="7"/>
-      <c r="J26" s="26"/>
-      <c r="K26" s="26"/>
-      <c r="L26" s="26"/>
-      <c r="M26" s="4"/>
-      <c r="N26" s="26"/>
-      <c r="O26" s="26"/>
-      <c r="P26" s="5"/>
-      <c r="Q26" s="6"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="21"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="10"/>
+      <c r="I26" s="11"/>
+      <c r="J26" s="9"/>
+      <c r="K26" s="12"/>
+      <c r="L26" s="9"/>
+      <c r="M26" s="13"/>
+      <c r="N26" s="13"/>
+      <c r="O26" s="8"/>
+      <c r="P26" s="8"/>
     </row>
-    <row r="27" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3"/>
       <c r="B27" s="1"/>
-      <c r="C27" s="19"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="25"/>
-      <c r="H27" s="25"/>
-      <c r="I27" s="7"/>
-      <c r="J27" s="26"/>
-      <c r="K27" s="26"/>
-      <c r="L27" s="26"/>
-      <c r="M27" s="4"/>
-      <c r="N27" s="26"/>
-      <c r="O27" s="26"/>
-      <c r="P27" s="5"/>
-      <c r="Q27" s="6"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="11"/>
+      <c r="J27" s="9"/>
+      <c r="K27" s="12"/>
+      <c r="L27" s="9"/>
+      <c r="M27" s="13"/>
+      <c r="N27" s="13"/>
+      <c r="O27" s="8"/>
+      <c r="P27" s="8"/>
     </row>
-    <row r="28" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3"/>
       <c r="B28" s="1"/>
       <c r="C28" s="8"/>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
-      <c r="F28" s="22"/>
+      <c r="F28" s="21"/>
       <c r="G28" s="10"/>
       <c r="H28" s="10"/>
       <c r="I28" s="11"/>
@@ -1187,54 +1149,15 @@
       <c r="L28" s="9"/>
       <c r="M28" s="13"/>
       <c r="N28" s="13"/>
-      <c r="O28" s="13"/>
+      <c r="O28" s="8"/>
       <c r="P28" s="8"/>
-      <c r="Q28" s="8"/>
     </row>
-    <row r="29" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="3"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="22"/>
-      <c r="G29" s="10"/>
-      <c r="H29" s="10"/>
-      <c r="I29" s="11"/>
-      <c r="J29" s="9"/>
-      <c r="K29" s="12"/>
-      <c r="L29" s="9"/>
-      <c r="M29" s="13"/>
-      <c r="N29" s="13"/>
-      <c r="O29" s="13"/>
-      <c r="P29" s="8"/>
-      <c r="Q29" s="8"/>
-    </row>
-    <row r="30" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="3"/>
-      <c r="B30" s="1"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
+    <row r="30" spans="1:16" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B30" s="20"/>
       <c r="F30" s="22"/>
-      <c r="G30" s="10"/>
-      <c r="H30" s="10"/>
-      <c r="I30" s="11"/>
-      <c r="J30" s="9"/>
-      <c r="K30" s="12"/>
-      <c r="L30" s="9"/>
-      <c r="M30" s="13"/>
-      <c r="N30" s="13"/>
-      <c r="O30" s="13"/>
-      <c r="P30" s="8"/>
-      <c r="Q30" s="8"/>
-    </row>
-    <row r="32" spans="1:17" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="B32" s="21"/>
-      <c r="F32" s="23"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
@@ -1248,7 +1171,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5546875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="26" width="10" customWidth="1"/>
   </cols>
@@ -2262,7 +2185,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5546875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="26" width="10" customWidth="1"/>
   </cols>

</xml_diff>